<commit_message>
feat: browser-free snapshots of the live Google Sheet
src/sheet_snapshots.py asks Google to render Dashboard and Inventory through
the spreadsheet PDF export endpoint (service-account auth), rasterises the
page with PyMuPDF and trims the margin - no browser automation involved.
visuals.py frames them as slides 02 and 05. Readable series/strategy labels
and tighter Inventory column widths in the sheet.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/out/07_Before_vs_After.xlsx
+++ b/out/07_Before_vs_After.xlsx
@@ -667,11 +667,11 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
-    <col width="30" customWidth="1" min="2" max="2"/>
-    <col width="29" customWidth="1" min="3" max="3"/>
-    <col width="28" customWidth="1" min="4" max="4"/>
-    <col width="28" customWidth="1" min="5" max="5"/>
-    <col width="26" customWidth="1" min="6" max="6"/>
+    <col width="22" customWidth="1" min="2" max="2"/>
+    <col width="23" customWidth="1" min="3" max="3"/>
+    <col width="23" customWidth="1" min="4" max="4"/>
+    <col width="23" customWidth="1" min="5" max="5"/>
+    <col width="18" customWidth="1" min="6" max="6"/>
     <col width="15" customWidth="1" min="7" max="7"/>
     <col width="23" customWidth="1" min="8" max="8"/>
     <col width="16" customWidth="1" min="9" max="9"/>
@@ -689,27 +689,27 @@
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
-          <t>oversold orders - sync 1440m</t>
+          <t>oversold: daily sync</t>
         </is>
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
-          <t>oversold orders - sync 240m</t>
+          <t>oversold: 4-hour sync</t>
         </is>
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
-          <t>oversold orders - sync 60m</t>
+          <t>oversold: hourly sync</t>
         </is>
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
-          <t>oversold orders - sync 15m</t>
+          <t>oversold: 15-min sync</t>
         </is>
       </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
-          <t>oversold orders - engine</t>
+          <t>oversold: engine</t>
         </is>
       </c>
       <c r="G1" s="1" t="inlineStr">

</xml_diff>